<commit_message>
Add 15 more pre-seed/early-stage VCs and accelerators
https://claude.ai/code/session_01VZSSJ5Wxbsq72rP35q9KHj
</commit_message>
<xml_diff>
--- a/korea_vc_list.xlsx
+++ b/korea_vc_list.xlsx
@@ -10,7 +10,7 @@
     <sheet name="한국 VC 리스트" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'한국 VC 리스트'!$A$1:$E$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'한국 VC 리스트'!$A$1:$E$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -901,399 +901,395 @@
       <c r="E15" s="2" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>초기~중기 (Series A/B)</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>알토스벤처스 (Altos Ventures)</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Series A~C</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>쿠팡·크래프톤 등 대형 투자, 미국계 독립 VC</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>altosvc.com</t>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>초기 (Pre-Seed/Seed)</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>블루포인트파트너스 (Bluepoint Partners)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Seed / Seed</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>이용관 설립, 딥테크 특화, 창업자 선호 1위 AC, 200개+ 투자</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>bluepoint.ac</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>초기~중기 (Series A/B)</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>소프트뱅크벤처스아시아</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Series A~C</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>소프트뱅크 계열, 아시아 특화</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>softbank.vc</t>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>초기 (Pre-Seed/Seed)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>소풍벤처스 (Sopoong Ventures)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Seed / Seed</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>임팩트·소셜벤처 특화, 2024년 VC 라이선스 취득</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>sopoong.net</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>초기~중기 (Series A/B)</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>IMM인베스트먼트</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Series A~C</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>대형 독립계 VC</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>imminvestment.com</t>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>초기 (Pre-Seed/Seed)</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>해시드 (Hashed)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Seed / Series A</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>블록체인·Web3 전문 글로벌 VC, 김서준 설립</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>hashed.com</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>초기~중기 (Series A/B)</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>한국투자파트너스</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Series A~C</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>한국투자증권 계열</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>kipvc.com</t>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>초기 (Pre-Seed/Seed)</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>캡스톤파트너스 (Capstone Partners)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Seed / Series A</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>독립계 초기 VC, 500억+ 펀드 운용</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>capstonepartners.co.kr</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>초기~중기 (Series A/B)</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>LB인베스트먼트</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Series A~C</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>LG그룹 계열 VC</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>lbinvestment.co.kr</t>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>초기 (Pre-Seed/Seed)</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>스트롱벤처스 (Strong Ventures)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Seed / Series A</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>미국·한국 크로스보더 초기 투자, 2025H1 11건 투자</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>strongvc.com</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>초기~중기 (Series A/B)</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>미래에셋벤처투자</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Series A~C</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>미래에셋 계열</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>miraeassetventure.com</t>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>초기 (Pre-Seed/Seed)</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>씨엔티테크 (CNT Tech)</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Seed / Seed</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>2003년 설립, 스포츠·엔터프라이즈 특화 AC, 상장 추진 중</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>cntt.co.kr</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>초기~중기 (Series A/B)</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>KB인베스트먼트</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Series A~C</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>KB금융 계열</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>kbinvestment.co.kr</t>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>초기 (Pre-Seed/Seed)</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>더인벤션랩 (The Invention Lab)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Seed / Seed</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>2014년 설립, 누적 투자 260억, 25개+ 펀드 운용, AI·딥테크</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>theinventionlab.co.kr</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>초기~중기 (Series A/B)</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>신한벤처투자</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Series A~C</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>신한금융 계열</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>shinhanventure.com</t>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>초기 (Pre-Seed/Seed)</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>빅뱅엔젤스 (BigBang Angels)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Seed / Seed</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>2012년 설립, 엔터프라이즈·B2B SaaS 특화 AC</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>bigbangangels.com</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>초기~중기 (Series A/B)</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>하나벤처스</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Series A~C</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>하나금융 계열</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>hanaventures.co.kr</t>
-        </is>
-      </c>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>초기 (Pre-Seed/Seed)</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>슈미트 (Schmidt)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Seed / Seed</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>2025H1 10건+ 투자, 초기 스타트업 특화 AC</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>초기~중기 (Series A/B)</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>인터베스트 (InterVest)</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Series A~C</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>독립계, IT·바이오 특화</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>intervest.co.kr</t>
-        </is>
-      </c>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>초기 (Pre-Seed/Seed)</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>엠와이소셜컴퍼니 (MY Social Company)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Seed / Seed</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>2025H1 초기 라운드 투자 최다 참여 AC 중 하나</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>초기~중기 (Series A/B)</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>스마일게이트인베스트먼트</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Series A~C</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>스마일게이트 CVC</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>초기 (Pre-Seed/Seed)</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>한국투자액셀러레이터</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Seed / Seed</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>한국투자증권 계열 AC, 검증된 금융 네트워크 보유</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>ac.koreainvestment.com</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>초기~중기 (Series A/B)</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>카카오인베스트먼트</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>Series A~C</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>카카오 계열 성장 투자</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr"/>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>초기 (Pre-Seed/Seed)</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>테크스타스 코리아 (Techstars Korea)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Seed / Seed</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>글로벌 액셀러레이터 Techstars 한국 프로그램</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>techstars.com</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>초기~중기 (Series A/B)</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>KDB산업은행 캐피탈</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>Series A~C</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>정책금융 기관</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>kdbcapital.co.kr</t>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>초기 (Pre-Seed/Seed)</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>K-Startup (정부 프로그램)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Seed / Seed</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>정부 지원 글로벌 스타트업 육성 프로그램, 중기부 운영</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>k-startup.go.kr</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>초기~중기 (Series A/B)</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>DSC인베스트먼트</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Series A~C</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>상장 독립계 VC</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>dscinvestment.com</t>
-        </is>
-      </c>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>초기 (Pre-Seed/Seed)</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>로아인벤션랩 (ROA Invention Lab)</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Seed / Seed</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>지능정보·AI 특화 AC, K-Global 액셀러레이터 육성사업 참여</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>초기~중기 (Series A/B)</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>SV인베스트먼트</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Series A~C</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>독립계 VC</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>svinvestment.co.kr</t>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>초기 (Pre-Seed/Seed)</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>한국엔젤투자협회 (KBAN)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Seed / Seed</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>2012년 설립, 엔젤투자 지원 및 매칭 플랫폼 운영</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>kban.or.kr</t>
         </is>
       </c>
     </row>
@@ -1305,620 +1301,1017 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
+          <t>알토스벤처스 (Altos Ventures)</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Series A~C</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>쿠팡·크래프톤 등 대형 투자, 미국계 독립 VC</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>altosvc.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>초기~중기 (Series A/B)</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>소프트뱅크벤처스아시아</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Series A~C</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>소프트뱅크 계열, 아시아 특화</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>softbank.vc</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>초기~중기 (Series A/B)</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>IMM인베스트먼트</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Series A~C</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>대형 독립계 VC</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>imminvestment.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>초기~중기 (Series A/B)</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>한국투자파트너스</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Series A~C</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>한국투자증권 계열</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>kipvc.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>초기~중기 (Series A/B)</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>LB인베스트먼트</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Series A~C</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>LG그룹 계열 VC</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>lbinvestment.co.kr</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>초기~중기 (Series A/B)</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>미래에셋벤처투자</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Series A~C</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>미래에셋 계열</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>miraeassetventure.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>초기~중기 (Series A/B)</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>KB인베스트먼트</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Series A~C</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>KB금융 계열</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>kbinvestment.co.kr</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>초기~중기 (Series A/B)</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>신한벤처투자</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Series A~C</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>신한금융 계열</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>shinhanventure.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>초기~중기 (Series A/B)</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>하나벤처스</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Series A~C</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>하나금융 계열</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>hanaventures.co.kr</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>초기~중기 (Series A/B)</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>인터베스트 (InterVest)</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Series A~C</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>독립계, IT·바이오 특화</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>intervest.co.kr</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>초기~중기 (Series A/B)</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>스마일게이트인베스트먼트</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Series A~C</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>스마일게이트 CVC</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>초기~중기 (Series A/B)</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>카카오인베스트먼트</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Series A~C</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>카카오 계열 성장 투자</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>초기~중기 (Series A/B)</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>KDB산업은행 캐피탈</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Series A~C</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>정책금융 기관</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>kdbcapital.co.kr</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>초기~중기 (Series A/B)</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>DSC인베스트먼트</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Series A~C</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>상장 독립계 VC</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>dscinvestment.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>초기~중기 (Series A/B)</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>SV인베스트먼트</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Series A~C</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>독립계 VC</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>svinvestment.co.kr</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>초기~중기 (Series A/B)</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
           <t>세마인베스트먼트</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>Series A~C</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>독립계 VC</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>semavc.com</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="6" t="inlineStr">
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>성장·후기 (Series B/C/Pre-IPO)</t>
         </is>
       </c>
-      <c r="B32" s="7" t="inlineStr">
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>스틱인베스트먼트 (STIC)</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>Series B~D</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>PE·VC 겸업, 대형 펀드 운용</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="E47" s="6" t="inlineStr">
         <is>
           <t>sticvc.com</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="6" t="inlineStr">
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>성장·후기 (Series B/C/Pre-IPO)</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B48" s="7" t="inlineStr">
         <is>
           <t>에이티넘인베스트먼트</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>Series B~D</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D48" s="6" t="inlineStr">
         <is>
           <t>대형 독립계 VC</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
+      <c r="E48" s="6" t="inlineStr">
         <is>
           <t>atinum.co.kr</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="6" t="inlineStr">
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="6" t="inlineStr">
         <is>
           <t>성장·후기 (Series B/C/Pre-IPO)</t>
         </is>
       </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="B49" s="7" t="inlineStr">
         <is>
           <t>UTC인베스트먼트</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>Series B~D</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>독립계, 제조·기술 특화</t>
         </is>
       </c>
-      <c r="E34" s="6" t="inlineStr">
+      <c r="E49" s="6" t="inlineStr">
         <is>
           <t>utcis.co.kr</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="6" t="inlineStr">
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>성장·후기 (Series B/C/Pre-IPO)</t>
         </is>
       </c>
-      <c r="B35" s="7" t="inlineStr">
+      <c r="B50" s="7" t="inlineStr">
         <is>
           <t>큐캐피탈파트너스</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C50" s="6" t="inlineStr">
         <is>
           <t>Series B~D</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr">
+      <c r="D50" s="6" t="inlineStr">
         <is>
           <t>PE·VC 겸업</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="E50" s="6" t="inlineStr">
         <is>
           <t>qcapital.co.kr</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="6" t="inlineStr">
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="6" t="inlineStr">
         <is>
           <t>성장·후기 (Series B/C/Pre-IPO)</t>
         </is>
       </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="B51" s="7" t="inlineStr">
         <is>
           <t>TS인베스트먼트</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>Series A~C</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>상장사, 바이오·IT 특화</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="E51" s="6" t="inlineStr">
         <is>
           <t>ts-investment.co.kr</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="6" t="inlineStr">
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>성장·후기 (Series B/C/Pre-IPO)</t>
         </is>
       </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="B52" s="7" t="inlineStr">
         <is>
           <t>한화인베스트먼트</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C52" s="6" t="inlineStr">
         <is>
           <t>Series B~D</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="D52" s="6" t="inlineStr">
         <is>
           <t>한화그룹 CVC</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr"/>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="6" t="inlineStr">
+      <c r="E52" s="6" t="inlineStr"/>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="6" t="inlineStr">
         <is>
           <t>성장·후기 (Series B/C/Pre-IPO)</t>
         </is>
       </c>
-      <c r="B38" s="7" t="inlineStr">
+      <c r="B53" s="7" t="inlineStr">
         <is>
           <t>신세계 시그나이트파트너스</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C53" s="6" t="inlineStr">
         <is>
           <t>Series A~C</t>
         </is>
       </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>신세계그룹 CVC</t>
         </is>
       </c>
-      <c r="E38" s="6" t="inlineStr">
+      <c r="E53" s="6" t="inlineStr">
         <is>
           <t>signiteventures.com</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="6" t="inlineStr">
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>성장·후기 (Series B/C/Pre-IPO)</t>
         </is>
       </c>
-      <c r="B39" s="7" t="inlineStr">
+      <c r="B54" s="7" t="inlineStr">
         <is>
           <t>GS벤처스</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C54" s="6" t="inlineStr">
         <is>
           <t>Series B~C</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D54" s="6" t="inlineStr">
         <is>
           <t>GS그룹 CVC</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr"/>
-    </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="6" t="inlineStr">
+      <c r="E54" s="6" t="inlineStr"/>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>성장·후기 (Series B/C/Pre-IPO)</t>
         </is>
       </c>
-      <c r="B40" s="7" t="inlineStr">
+      <c r="B55" s="7" t="inlineStr">
         <is>
           <t>CJ인베스트먼트</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>Series A~C</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>CJ그룹 CVC</t>
         </is>
       </c>
-      <c r="E40" s="6" t="inlineStr"/>
-    </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="6" t="inlineStr">
+      <c r="E55" s="6" t="inlineStr"/>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>성장·후기 (Series B/C/Pre-IPO)</t>
         </is>
       </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="B56" s="7" t="inlineStr">
         <is>
           <t>롯데벤처스</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
+      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>Series A~C</t>
         </is>
       </c>
-      <c r="D41" s="6" t="inlineStr">
+      <c r="D56" s="6" t="inlineStr">
         <is>
           <t>롯데그룹 CVC</t>
         </is>
       </c>
-      <c r="E41" s="6" t="inlineStr"/>
-    </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="6" t="inlineStr">
+      <c r="E56" s="6" t="inlineStr"/>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="6" t="inlineStr">
         <is>
           <t>성장·후기 (Series B/C/Pre-IPO)</t>
         </is>
       </c>
-      <c r="B42" s="7" t="inlineStr">
+      <c r="B57" s="7" t="inlineStr">
         <is>
           <t>크레비스파트너스</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>Series A~C</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="D57" s="6" t="inlineStr">
         <is>
           <t>임팩트·사회적 가치 투자</t>
         </is>
       </c>
-      <c r="E42" s="6" t="inlineStr">
+      <c r="E57" s="6" t="inlineStr">
         <is>
           <t>crevisse.com</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="6" t="inlineStr">
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="6" t="inlineStr">
         <is>
           <t>성장·후기 (Series B/C/Pre-IPO)</t>
         </is>
       </c>
-      <c r="B43" s="7" t="inlineStr">
+      <c r="B58" s="7" t="inlineStr">
         <is>
           <t>위벤처스 (We Ventures)</t>
         </is>
       </c>
-      <c r="C43" s="6" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>Series A~C</t>
         </is>
       </c>
-      <c r="D43" s="6" t="inlineStr">
+      <c r="D58" s="6" t="inlineStr">
         <is>
           <t>여성 창업자·다양성 강조</t>
         </is>
       </c>
-      <c r="E43" s="6" t="inlineStr">
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>we.vc</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="6" t="inlineStr">
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="6" t="inlineStr">
         <is>
           <t>성장·후기 (Series B/C/Pre-IPO)</t>
         </is>
       </c>
-      <c r="B44" s="7" t="inlineStr">
+      <c r="B59" s="7" t="inlineStr">
         <is>
           <t>스퀘어원파트너스</t>
         </is>
       </c>
-      <c r="C44" s="6" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>Series A~C</t>
         </is>
       </c>
-      <c r="D44" s="6" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>핀테크·SaaS 특화</t>
         </is>
       </c>
-      <c r="E44" s="6" t="inlineStr"/>
-    </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="6" t="inlineStr">
+      <c r="E59" s="6" t="inlineStr"/>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="6" t="inlineStr">
         <is>
           <t>성장·후기 (Series B/C/Pre-IPO)</t>
         </is>
       </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="B60" s="7" t="inlineStr">
         <is>
           <t>NH농협PE</t>
         </is>
       </c>
-      <c r="C45" s="6" t="inlineStr">
+      <c r="C60" s="6" t="inlineStr">
         <is>
           <t>Series B~D</t>
         </is>
       </c>
-      <c r="D45" s="6" t="inlineStr">
+      <c r="D60" s="6" t="inlineStr">
         <is>
           <t>NH농협금융 계열</t>
         </is>
       </c>
-      <c r="E45" s="6" t="inlineStr"/>
-    </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="E60" s="6" t="inlineStr"/>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="8" t="inlineStr">
         <is>
           <t>글로벌·크로스보더</t>
         </is>
       </c>
-      <c r="B46" s="9" t="inlineStr">
+      <c r="B61" s="9" t="inlineStr">
         <is>
           <t>알토스벤처스 (Altos Ventures)</t>
         </is>
       </c>
-      <c r="C46" s="8" t="inlineStr">
+      <c r="C61" s="8" t="inlineStr">
         <is>
           <t>Series A~C+</t>
         </is>
       </c>
-      <c r="D46" s="8" t="inlineStr">
+      <c r="D61" s="8" t="inlineStr">
         <is>
           <t>미국 본사, 한국 스타트업 집중 투자</t>
         </is>
       </c>
-      <c r="E46" s="8" t="inlineStr">
+      <c r="E61" s="8" t="inlineStr">
         <is>
           <t>altosvc.com</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="8" t="inlineStr">
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>글로벌·크로스보더</t>
         </is>
       </c>
-      <c r="B47" s="9" t="inlineStr">
+      <c r="B62" s="9" t="inlineStr">
         <is>
           <t>소프트뱅크벤처스아시아</t>
         </is>
       </c>
-      <c r="C47" s="8" t="inlineStr">
+      <c r="C62" s="8" t="inlineStr">
         <is>
           <t>Series B~C</t>
         </is>
       </c>
-      <c r="D47" s="8" t="inlineStr">
+      <c r="D62" s="8" t="inlineStr">
         <is>
           <t>일본 소프트뱅크 계열, 아시아 투자</t>
         </is>
       </c>
-      <c r="E47" s="8" t="inlineStr">
+      <c r="E62" s="8" t="inlineStr">
         <is>
           <t>softbank.vc</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="8" t="inlineStr">
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="8" t="inlineStr">
         <is>
           <t>글로벌·크로스보더</t>
         </is>
       </c>
-      <c r="B48" s="9" t="inlineStr">
+      <c r="B63" s="9" t="inlineStr">
         <is>
           <t>500 스타트업스 코리아</t>
         </is>
       </c>
-      <c r="C48" s="8" t="inlineStr">
+      <c r="C63" s="8" t="inlineStr">
         <is>
           <t>Seed~Series A</t>
         </is>
       </c>
-      <c r="D48" s="8" t="inlineStr">
+      <c r="D63" s="8" t="inlineStr">
         <is>
           <t>글로벌 액셀러레이터 한국 프로그램</t>
         </is>
       </c>
-      <c r="E48" s="8" t="inlineStr"/>
-    </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="E63" s="8" t="inlineStr"/>
+    </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>글로벌·크로스보더</t>
         </is>
       </c>
-      <c r="B49" s="9" t="inlineStr">
+      <c r="B64" s="9" t="inlineStr">
         <is>
           <t>스파크랩 글로벌</t>
         </is>
       </c>
-      <c r="C49" s="8" t="inlineStr">
+      <c r="C64" s="8" t="inlineStr">
         <is>
           <t>Seed~Series A</t>
         </is>
       </c>
-      <c r="D49" s="8" t="inlineStr">
+      <c r="D64" s="8" t="inlineStr">
         <is>
           <t>미국·한국 연결 액셀러레이터</t>
         </is>
       </c>
-      <c r="E49" s="8" t="inlineStr">
+      <c r="E64" s="8" t="inlineStr">
         <is>
           <t>sparklabs.co.kr</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="8" t="inlineStr">
+    <row r="65" ht="18" customHeight="1">
+      <c r="A65" s="8" t="inlineStr">
         <is>
           <t>글로벌·크로스보더</t>
         </is>
       </c>
-      <c r="B50" s="9" t="inlineStr">
+      <c r="B65" s="9" t="inlineStr">
         <is>
           <t>블루런벤처스 (BlueRun)</t>
         </is>
       </c>
-      <c r="C50" s="8" t="inlineStr">
+      <c r="C65" s="8" t="inlineStr">
         <is>
           <t>Series A~C</t>
         </is>
       </c>
-      <c r="D50" s="8" t="inlineStr">
+      <c r="D65" s="8" t="inlineStr">
         <is>
           <t>미국계, 모바일·인터넷 특화</t>
         </is>
       </c>
-      <c r="E50" s="8" t="inlineStr">
+      <c r="E65" s="8" t="inlineStr">
         <is>
           <t>brv.com</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="10" t="inlineStr">
+    <row r="66" ht="18" customHeight="1">
+      <c r="A66" s="10" t="inlineStr">
         <is>
           <t>정책 기관</t>
         </is>
       </c>
-      <c r="B51" s="11" t="inlineStr">
+      <c r="B66" s="11" t="inlineStr">
         <is>
           <t>한국벤처투자 (KVIC)</t>
         </is>
       </c>
-      <c r="C51" s="10" t="inlineStr">
+      <c r="C66" s="10" t="inlineStr">
         <is>
           <t>모태펀드 출자</t>
         </is>
       </c>
-      <c r="D51" s="10" t="inlineStr">
+      <c r="D66" s="10" t="inlineStr">
         <is>
           <t>모태펀드 운용, 전체 VC 출자 기관</t>
         </is>
       </c>
-      <c r="E51" s="10" t="inlineStr">
+      <c r="E66" s="10" t="inlineStr">
         <is>
           <t>kvic.or.kr</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="10" t="inlineStr">
+    <row r="67" ht="18" customHeight="1">
+      <c r="A67" s="10" t="inlineStr">
         <is>
           <t>정책 기관</t>
         </is>
       </c>
-      <c r="B52" s="11" t="inlineStr">
+      <c r="B67" s="11" t="inlineStr">
         <is>
           <t>기술보증기금 (KIBO)</t>
         </is>
       </c>
-      <c r="C52" s="10" t="inlineStr">
+      <c r="C67" s="10" t="inlineStr">
         <is>
           <t>Seed~Series A</t>
         </is>
       </c>
-      <c r="D52" s="10" t="inlineStr">
+      <c r="D67" s="10" t="inlineStr">
         <is>
           <t>기술 창업 보증·투자</t>
         </is>
       </c>
-      <c r="E52" s="10" t="inlineStr">
+      <c r="E67" s="10" t="inlineStr">
         <is>
           <t>kibo.or.kr</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="10" t="inlineStr">
+    <row r="68" ht="18" customHeight="1">
+      <c r="A68" s="10" t="inlineStr">
         <is>
           <t>정책 기관</t>
         </is>
       </c>
-      <c r="B53" s="11" t="inlineStr">
+      <c r="B68" s="11" t="inlineStr">
         <is>
           <t>신용보증기금</t>
         </is>
       </c>
-      <c r="C53" s="10" t="inlineStr">
+      <c r="C68" s="10" t="inlineStr">
         <is>
           <t>Seed~Series A</t>
         </is>
       </c>
-      <c r="D53" s="10" t="inlineStr">
+      <c r="D68" s="10" t="inlineStr">
         <is>
           <t>스타트업 보증 지원</t>
         </is>
       </c>
-      <c r="E53" s="10" t="inlineStr">
+      <c r="E68" s="10" t="inlineStr">
         <is>
           <t>kodit.co.kr</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="10" t="inlineStr">
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="10" t="inlineStr">
         <is>
           <t>정책 기관</t>
         </is>
       </c>
-      <c r="B54" s="11" t="inlineStr">
+      <c r="B69" s="11" t="inlineStr">
         <is>
           <t>TIPS 프로그램 (중기부)</t>
         </is>
       </c>
-      <c r="C54" s="10" t="inlineStr">
+      <c r="C69" s="10" t="inlineStr">
         <is>
           <t>Seed~Series A</t>
         </is>
       </c>
-      <c r="D54" s="10" t="inlineStr">
+      <c r="D69" s="10" t="inlineStr">
         <is>
           <t>민간 투자 주도형 기술 창업 지원</t>
         </is>
       </c>
-      <c r="E54" s="10" t="inlineStr">
+      <c r="E69" s="10" t="inlineStr">
         <is>
           <t>jointips.or.kr</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E54"/>
+  <autoFilter ref="A1:E69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>